<commit_message>
Importação com foto do produto (coluna imagem), planilha-modelo atualizada; marca do demo configurável (brand.json)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TPoeb89LuaKuSd6trTc9C8
</commit_message>
<xml_diff>
--- a/docs/geolynq-catalogo-modelo.xlsx
+++ b/docs/geolynq-catalogo-modelo.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Produtos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Revendedores" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Cobertura" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Produtos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revendedores" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -151,6 +151,21 @@
     <author>GeoLynq</author>
   </authors>
   <commentList>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Opcional. Link da foto do produto, começando com https:// (até 500 caracteres, sem espaços). Vazio = produto sem foto (o widget mostra as iniciais). Link com http:// ou com espaço é ignorado e aparece como AVISO na importação.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>GeoLynq</author>
+  </authors>
+  <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
         <t>CNPJ do revendedor, 14 dígitos (pode ter pontos e traço). OBRIGATÓRIO para cliente novo: é a chave que impede duplicar o revendedor ao reimportar. Deixe esta coluna no formato Texto, senão o Excel/Sheets apaga o zero à esquerda. Rede com várias lojas: um CNPJ por loja (final 0001, 0002...).</t>
@@ -165,7 +180,7 @@
 </comments>
 </file>
 
-<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>GeoLynq</author>
@@ -469,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -477,6 +492,7 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -505,6 +521,11 @@
           <t>alergenos</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>imagem</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -532,9 +553,15 @@
           <t>leite</t>
         </is>
       </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.seusite.com.br/imagens/wpi-900.jpg</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>